<commit_message>
docs: reconcile submission artifacts and spreadsheet summary
</commit_message>
<xml_diff>
--- a/submit/23127326_test-cases.xlsx
+++ b/submit/23127326_test-cases.xlsx
@@ -199,7 +199,7 @@
       </c>
       <c r="B7" s="1">
         <f>COUNTA('Test Cases'!$A$2:$A$141)</f>
-        <v/>
+        <v>140</v>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
@@ -208,7 +208,7 @@
       </c>
       <c r="E7" s="1">
         <f>COUNTIF('Test Cases'!$B$2:$B$141,D7)</f>
-        <v/>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -219,7 +219,7 @@
       </c>
       <c r="B8" s="1">
         <f>COUNTIF('Test Cases'!$T$2:$T$141,"PASS")</f>
-        <v/>
+        <v>98</v>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
@@ -228,7 +228,7 @@
       </c>
       <c r="E8" s="1">
         <f>COUNTIF('Test Cases'!$B$2:$B$141,D8)</f>
-        <v/>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -239,7 +239,7 @@
       </c>
       <c r="B9" s="1">
         <f>COUNTIF('Test Cases'!$R$2:$R$141,"FAIL")</f>
-        <v/>
+        <v>42</v>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
@@ -248,7 +248,7 @@
       </c>
       <c r="E9" s="1">
         <f>COUNTIF('Test Cases'!$B$2:$B$141,D9)</f>
-        <v/>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -259,7 +259,7 @@
       </c>
       <c r="B10" s="1">
         <f>COUNTIF('Test Cases'!$T$2:$T$141,"PRODUCT DEFECT")</f>
-        <v/>
+        <v>42</v>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
@@ -268,7 +268,7 @@
       </c>
       <c r="E10" s="1">
         <f>SUM(E7:E9)</f>
-        <v/>
+        <v>140</v>
       </c>
     </row>
     <row r="11"/>
@@ -315,7 +315,7 @@
       </c>
       <c r="B15" s="1">
         <f>COUNTIF('Test Cases'!$L$2:$L$141,A15)</f>
-        <v/>
+        <v>125</v>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
@@ -324,7 +324,7 @@
       </c>
       <c r="E15" s="1">
         <f>COUNTIF('Test Cases'!$M$2:$M$141,D15)</f>
-        <v/>
+        <v>140</v>
       </c>
     </row>
     <row r="16">
@@ -335,7 +335,7 @@
       </c>
       <c r="B16" s="1">
         <f>COUNTIF('Test Cases'!$L$2:$L$141,A16)</f>
-        <v/>
+        <v>15</v>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
@@ -344,7 +344,7 @@
       </c>
       <c r="E16" s="1">
         <f>COUNTIF('Test Cases'!$M$2:$M$141,"&lt;&gt;VALID")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -355,7 +355,7 @@
       </c>
       <c r="B17" s="1">
         <f>SUM(B15:B16)</f>
-        <v/>
+        <v>140</v>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
@@ -364,7 +364,7 @@
       </c>
       <c r="E17" s="1">
         <f>SUM(E15:E16)</f>
-        <v/>
+        <v>140</v>
       </c>
     </row>
     <row r="18"/>

</xml_diff>

<commit_message>
docs: add comprehensive commit log for submission artifacts and updates
- Added PDF versions of various reports including README, AI audit, critique, bug reports, CI/CD, and main report.
- Reconciled submission artifacts with spreadsheet summary, updating test cases and documentation.
- Updated README and reports, added video demo, and bug report.
- Introduced CI configuration for submission.
- Finalized API testing submission package, including updates to commit logs and documentation.
- Renamed submission artifacts to include student ID for clarity.
- Moved reports to the root of the submission directory for better accessibility.
- Documented evidence of CI runs and linked verified GitHub bug issues.
- Added screenshots and evidence for CI and Newman executions.
- Recorded final commit log and ensured all documentation is up to date.
</commit_message>
<xml_diff>
--- a/submit/23127326_test-cases.xlsx
+++ b/submit/23127326_test-cases.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="L3" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M3" s="1" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="L4" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M4" s="1" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="L5" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M5" s="1" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="L6" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M6" s="1" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="L7" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M7" s="1" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="L8" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M8" s="1" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="L9" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M9" s="1" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="L10" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M10" s="1" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="L11" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M11" s="1" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="L12" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M12" s="1" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="L13" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M13" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="L14" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M14" s="1" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="L15" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M15" s="1" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="L16" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M16" s="1" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="L17" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M17" s="1" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="L18" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M18" s="1" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="L19" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M19" s="1" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="L20" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M20" s="1" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="L21" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M21" s="1" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="L22" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M22" s="1" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="L23" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M23" s="1" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="L24" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M24" s="1" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="L25" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M25" s="1" t="inlineStr">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="L26" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M26" s="1" t="inlineStr">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="L27" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M27" s="1" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="L28" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M28" s="1" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="L29" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M29" s="1" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="L30" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M30" s="1" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="L31" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M31" s="1" t="inlineStr">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="L32" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M32" s="1" t="inlineStr">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="L33" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M33" s="1" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="L34" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M34" s="1" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="L35" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M35" s="1" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="L36" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M36" s="1" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="L37" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M37" s="1" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="L38" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M38" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="L39" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M39" s="1" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="L40" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M40" s="1" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="L41" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-002</t>
         </is>
       </c>
       <c r="M41" s="1" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="L47" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M47" s="1" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="L48" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M48" s="1" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="L49" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M49" s="1" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="L50" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M50" s="1" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="L51" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M51" s="1" t="inlineStr">
@@ -5788,7 +5788,7 @@
       </c>
       <c r="L52" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M52" s="1" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="L53" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M53" s="1" t="inlineStr">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="L54" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M54" s="1" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="L55" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M55" s="1" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="L56" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M56" s="1" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="L57" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M57" s="1" t="inlineStr">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="L58" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M58" s="1" t="inlineStr">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="L59" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M59" s="1" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="L60" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M60" s="1" t="inlineStr">
@@ -6706,7 +6706,7 @@
       </c>
       <c r="L61" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M61" s="1" t="inlineStr">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="L62" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M62" s="1" t="inlineStr">
@@ -6910,7 +6910,7 @@
       </c>
       <c r="L63" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M63" s="1" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="L64" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M64" s="1" t="inlineStr">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="L65" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M65" s="1" t="inlineStr">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="L66" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M66" s="1" t="inlineStr">
@@ -7318,7 +7318,7 @@
       </c>
       <c r="L67" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M67" s="1" t="inlineStr">
@@ -7420,7 +7420,7 @@
       </c>
       <c r="L68" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M68" s="1" t="inlineStr">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="L69" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M69" s="1" t="inlineStr">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="L70" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M70" s="1" t="inlineStr">
@@ -7731,7 +7731,7 @@
       </c>
       <c r="L71" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M71" s="1" t="inlineStr">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="L72" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M72" s="1" t="inlineStr">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="L73" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M73" s="1" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="L74" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M74" s="1" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="L75" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M75" s="1" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="L76" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M76" s="1" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="L77" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M77" s="1" t="inlineStr">
@@ -8450,7 +8450,7 @@
       </c>
       <c r="L78" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M78" s="1" t="inlineStr">
@@ -8552,7 +8552,7 @@
       </c>
       <c r="L79" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M79" s="1" t="inlineStr">
@@ -8654,7 +8654,7 @@
       </c>
       <c r="L80" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M80" s="1" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="L81" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M81" s="1" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="L82" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M82" s="1" t="inlineStr">
@@ -8965,7 +8965,7 @@
       </c>
       <c r="L83" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M83" s="1" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="L84" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M84" s="1" t="inlineStr">
@@ -9169,7 +9169,7 @@
       </c>
       <c r="L85" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M85" s="1" t="inlineStr">
@@ -9271,7 +9271,7 @@
       </c>
       <c r="L86" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M86" s="1" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="L87" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M87" s="1" t="inlineStr">
@@ -9475,7 +9475,7 @@
       </c>
       <c r="L88" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M88" s="1" t="inlineStr">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="L89" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M89" s="1" t="inlineStr">
@@ -9679,7 +9679,7 @@
       </c>
       <c r="L90" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M90" s="1" t="inlineStr">
@@ -9781,7 +9781,7 @@
       </c>
       <c r="L91" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-003</t>
         </is>
       </c>
       <c r="M91" s="1" t="inlineStr">
@@ -10423,7 +10423,7 @@
       </c>
       <c r="L97" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M97" s="1" t="inlineStr">
@@ -10525,7 +10525,7 @@
       </c>
       <c r="L98" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M98" s="1" t="inlineStr">
@@ -10627,7 +10627,7 @@
       </c>
       <c r="L99" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M99" s="1" t="inlineStr">
@@ -10729,7 +10729,7 @@
       </c>
       <c r="L100" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M100" s="1" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="L101" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M101" s="1" t="inlineStr">
@@ -10938,7 +10938,7 @@
       </c>
       <c r="L102" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M102" s="1" t="inlineStr">
@@ -11040,7 +11040,7 @@
       </c>
       <c r="L103" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M103" s="1" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="L104" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M104" s="1" t="inlineStr">
@@ -11244,7 +11244,7 @@
       </c>
       <c r="L105" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M105" s="1" t="inlineStr">
@@ -11346,7 +11346,7 @@
       </c>
       <c r="L106" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M106" s="1" t="inlineStr">
@@ -11448,7 +11448,7 @@
       </c>
       <c r="L107" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M107" s="1" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="L108" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M108" s="1" t="inlineStr">
@@ -11652,7 +11652,7 @@
       </c>
       <c r="L109" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M109" s="1" t="inlineStr">
@@ -11754,7 +11754,7 @@
       </c>
       <c r="L110" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M110" s="1" t="inlineStr">
@@ -11856,7 +11856,7 @@
       </c>
       <c r="L111" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M111" s="1" t="inlineStr">
@@ -11958,7 +11958,7 @@
       </c>
       <c r="L112" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M112" s="1" t="inlineStr">
@@ -12060,7 +12060,7 @@
       </c>
       <c r="L113" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M113" s="1" t="inlineStr">
@@ -12167,7 +12167,7 @@
       </c>
       <c r="L114" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M114" s="1" t="inlineStr">
@@ -12274,7 +12274,7 @@
       </c>
       <c r="L115" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M115" s="1" t="inlineStr">
@@ -12381,7 +12381,7 @@
       </c>
       <c r="L116" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M116" s="1" t="inlineStr">
@@ -12488,7 +12488,7 @@
       </c>
       <c r="L117" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M117" s="1" t="inlineStr">
@@ -12595,7 +12595,7 @@
       </c>
       <c r="L118" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M118" s="1" t="inlineStr">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="L119" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M119" s="1" t="inlineStr">
@@ -12809,7 +12809,7 @@
       </c>
       <c r="L120" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M120" s="1" t="inlineStr">
@@ -12916,7 +12916,7 @@
       </c>
       <c r="L121" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M121" s="1" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="L122" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M122" s="1" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="L123" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M123" s="1" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="L124" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M124" s="1" t="inlineStr">
@@ -13334,7 +13334,7 @@
       </c>
       <c r="L125" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M125" s="1" t="inlineStr">
@@ -13441,7 +13441,7 @@
       </c>
       <c r="L126" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M126" s="1" t="inlineStr">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="L127" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M127" s="1" t="inlineStr">
@@ -13650,7 +13650,7 @@
       </c>
       <c r="L128" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M128" s="1" t="inlineStr">
@@ -13752,7 +13752,7 @@
       </c>
       <c r="L129" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M129" s="1" t="inlineStr">
@@ -13859,7 +13859,7 @@
       </c>
       <c r="L130" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M130" s="1" t="inlineStr">
@@ -13961,7 +13961,7 @@
       </c>
       <c r="L131" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M131" s="1" t="inlineStr">
@@ -14068,7 +14068,7 @@
       </c>
       <c r="L132" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M132" s="1" t="inlineStr">
@@ -14175,7 +14175,7 @@
       </c>
       <c r="L133" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M133" s="1" t="inlineStr">
@@ -14282,7 +14282,7 @@
       </c>
       <c r="L134" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M134" s="1" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="L135" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M135" s="1" t="inlineStr">
@@ -14491,7 +14491,7 @@
       </c>
       <c r="L136" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-004</t>
         </is>
       </c>
       <c r="M136" s="1" t="inlineStr">

</xml_diff>

<commit_message>
docs: fix inconsistency in report
</commit_message>
<xml_diff>
--- a/submit/23127326_test-cases.xlsx
+++ b/submit/23127326_test-cases.xlsx
@@ -310,11 +310,11 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>AI-001</t>
+          <t>AI-generated (AI-002/003/004)</t>
         </is>
       </c>
       <c r="B15" s="1">
-        <f>COUNTIF('Test Cases'!$L$2:$L$141,A15)</f>
+        <f>COUNTIF('Test Cases'!$L$2:$L$141,"AI-002")+COUNTIF('Test Cases'!$L$2:$L$141,"AI-003")+COUNTIF('Test Cases'!$L$2:$L$141,"AI-004")</f>
         <v>125</v>
       </c>
       <c r="D15" s="1" t="inlineStr">

</xml_diff>